<commit_message>
new layout and options
</commit_message>
<xml_diff>
--- a/Caloris.xlsx
+++ b/Caloris.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jarygau\Desktop\Caloris\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1828683B-FE94-4040-9367-89B2B23A447A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D007908-E6C3-4A4B-8D72-D30240333EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="READ ME" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="61">
   <si>
     <t>Caloris</t>
   </si>
@@ -112,9 +112,6 @@
     <t>heat_input</t>
   </si>
   <si>
-    <t>material</t>
-  </si>
-  <si>
     <t>mass</t>
   </si>
   <si>
@@ -184,9 +181,6 @@
     <t>Uranium</t>
   </si>
   <si>
-    <t>contact</t>
-  </si>
-  <si>
     <t>solver type</t>
   </si>
   <si>
@@ -218,6 +212,15 @@
   </si>
   <si>
     <t>Iterations</t>
+  </si>
+  <si>
+    <t>material_conductivity</t>
+  </si>
+  <si>
+    <t>material_specific_heat</t>
+  </si>
+  <si>
+    <t>convection</t>
   </si>
 </sst>
 </file>
@@ -844,7 +847,9 @@
   <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="7" width="11.5703125" style="17" customWidth="1"/>
+    <col min="1" max="5" width="11.5703125" style="17" customWidth="1"/>
+    <col min="6" max="6" width="19.5703125" style="17" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" style="17" customWidth="1"/>
     <col min="8" max="16384" width="11.5703125" style="17"/>
   </cols>
   <sheetData>
@@ -865,13 +870,13 @@
         <v>23</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -879,10 +884,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>27</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>28</v>
       </c>
       <c r="D2" s="11">
         <v>273</v>
@@ -897,10 +902,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>29</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>30</v>
       </c>
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
@@ -916,10 +921,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>31</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>32</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
@@ -932,10 +937,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D5" s="11">
         <f>30+273</f>
@@ -1153,18 +1158,18 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <conditionalFormatting sqref="D2:D22">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="11" priority="3">
       <formula>C2&lt;&gt;"Thermostat"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H22">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>C2&lt;&gt;"Heater"</formula>
+  <conditionalFormatting sqref="E2:E22">
+    <cfRule type="expression" dxfId="10" priority="1">
+      <formula>C2&lt;&gt;"Node"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E22">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>C2&lt;&gt;"Node"</formula>
+  <conditionalFormatting sqref="H2:H22">
+    <cfRule type="expression" dxfId="9" priority="2">
+      <formula>C2&lt;&gt;"Heater"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -1191,49 +1196,50 @@
   <dimension ref="A1:M27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="7" width="11.5703125" style="19" customWidth="1"/>
+    <col min="1" max="6" width="11.5703125" style="19" customWidth="1"/>
+    <col min="7" max="7" width="18.42578125" style="19" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="11.5703125" style="19"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="M1" s="9" t="s">
         <v>44</v>
-      </c>
-      <c r="M1" s="9" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1247,7 +1253,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E2" s="18">
         <v>0.02</v>
@@ -1255,8 +1261,8 @@
       <c r="F2" s="11">
         <v>10</v>
       </c>
-      <c r="G2" s="12" t="s">
-        <v>47</v>
+      <c r="G2" s="12">
+        <v>28</v>
       </c>
       <c r="H2" s="13"/>
       <c r="I2" s="11"/>
@@ -1276,7 +1282,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E3" s="18">
         <v>0.02</v>
@@ -1285,7 +1291,7 @@
         <v>10</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H3" s="13"/>
       <c r="I3" s="11"/>
@@ -1305,7 +1311,7 @@
         <v>3</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="E4" s="18"/>
       <c r="F4" s="11">
@@ -1713,60 +1719,57 @@
       <c r="M27" s="11"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <conditionalFormatting sqref="E2:E27">
-    <cfRule type="expression" dxfId="11" priority="3">
-      <formula>OR(D2="radiation",D2="",D2="contact")</formula>
+    <cfRule type="expression" dxfId="8" priority="3">
+      <formula>OR(D2="radiation",D2="",D2="convection")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F27">
-    <cfRule type="expression" dxfId="10" priority="2">
+    <cfRule type="expression" dxfId="7" priority="2">
       <formula>OR(D2="radiation",D2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G27">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>D2&lt;&gt;"conduction"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H27">
-    <cfRule type="expression" dxfId="8" priority="10">
-      <formula>D2&lt;&gt;"contact"</formula>
+    <cfRule type="expression" dxfId="5" priority="10">
+      <formula>D2&lt;&gt;"convection"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:I27">
-    <cfRule type="expression" dxfId="7" priority="9">
+    <cfRule type="expression" dxfId="4" priority="9">
       <formula>D2&lt;&gt;"radiation"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J27">
-    <cfRule type="expression" dxfId="6" priority="8">
+    <cfRule type="expression" dxfId="3" priority="8">
       <formula>D2&lt;&gt;"radiation"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:K27">
-    <cfRule type="expression" dxfId="5" priority="7">
+    <cfRule type="expression" dxfId="2" priority="7">
       <formula>D2&lt;&gt;"radiation"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:L27">
-    <cfRule type="expression" dxfId="4" priority="6">
+    <cfRule type="expression" dxfId="1" priority="6">
       <formula>D2&lt;&gt;"radiation"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M27">
-    <cfRule type="expression" dxfId="3" priority="5">
+    <cfRule type="expression" dxfId="0" priority="5">
       <formula>D2&lt;&gt;"radiation"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" operator="equal" allowBlank="1" showErrorMessage="1" sqref="D2:D27" xr:uid="{00000000-0002-0000-0200-000000000000}">
-      <formula1>"conduction,radiation,direct_G,contact"</formula1>
-      <formula2>0</formula2>
+      <formula1>"conduction,radiation,conductance,convection"</formula1>
     </dataValidation>
-    <dataValidation type="list" operator="equal" allowBlank="1" showErrorMessage="1" sqref="G2:G27" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" operator="equal" allowBlank="1" sqref="G2:G27" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"Al6061,Al6063,CuRRR100,SST304L,Uranium"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
@@ -1799,29 +1802,29 @@
   <sheetData>
     <row r="5" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" t="s">
         <v>53</v>
-      </c>
-      <c r="B7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C7" t="s">
-        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1851,15 +1854,15 @@
   <sheetData>
     <row r="11" spans="7:8" x14ac:dyDescent="0.2">
       <c r="G11" s="21" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H11" s="21" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="7:8" x14ac:dyDescent="0.2">
       <c r="G12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H12" t="b">
         <v>1</v>
@@ -1867,7 +1870,7 @@
     </row>
     <row r="13" spans="7:8" x14ac:dyDescent="0.2">
       <c r="G13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H13">
         <v>26</v>

</xml_diff>